<commit_message>
Integration of cvxlab output into add_sector
First draft of integration of cvxlab output database into MARIO tables. Specific function for 'Split_sectors' case, still generic for other cases.
To be polished.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/mapping.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/mapping.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45DE26F3-0B93-4177-BE9C-9EF9840F4988}"/>
+  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB155895-4DD4-420C-A568-B817D6686D14}"/>
   <bookViews>
-    <workbookView xWindow="-8920" yWindow="-20500" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4785" yWindow="2940" windowWidth="19290" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
     <sheet name="matrices" sheetId="4" r:id="rId2"/>
-    <sheet name="matrices_old" sheetId="6" r:id="rId3"/>
+    <sheet name="matrices_old" sheetId="8" r:id="rId3"/>
+    <sheet name="result matrices" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t>sector_from</t>
   </si>
@@ -137,6 +138,33 @@
   </si>
   <si>
     <t>cons_categ</t>
+  </si>
+  <si>
+    <t>Znew_supply</t>
+  </si>
+  <si>
+    <t>Znew_use</t>
+  </si>
+  <si>
+    <t>Ynew</t>
+  </si>
+  <si>
+    <t>indeces</t>
+  </si>
+  <si>
+    <t>unstack</t>
+  </si>
+  <si>
+    <t>region_from_Name, sector_from_Name, region_to_Name, sector_to_Name</t>
+  </si>
+  <si>
+    <t>region_from_Name, sector_from_Name, region_to_Name, cons_categ_Name</t>
+  </si>
+  <si>
+    <t>region_to_Name, cons_categ_Name</t>
+  </si>
+  <si>
+    <t>region_to_Name, sector_to_Name</t>
   </si>
 </sst>
 </file>
@@ -193,11 +221,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,14 +530,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" customWidth="1"/>
-    <col min="3" max="3" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -519,7 +548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -530,7 +559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -541,7 +570,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -552,7 +581,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -563,7 +592,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -574,7 +603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -585,7 +614,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -596,7 +625,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -615,9 +644,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81EB35F2-9F14-A44D-AA1B-E427820E5706}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -628,7 +657,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -639,7 +668,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -650,7 +679,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -661,7 +690,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -678,11 +707,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D82ADD-CF17-4AD8-8471-E054155EA861}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212F1892-DFA1-4A7F-B6A7-3C40EACDE056}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -693,7 +722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -704,7 +733,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -713,6 +742,72 @@
       </c>
       <c r="C3" t="s">
         <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2E9369E-B0C1-4C05-9A69-D044DE2827CA}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tolerance definition from inventory
Tolerance for disaggregation routines can be defined by the user in the add_sectors inventory, a new sheet was created. There is a problem with the export of the split matrices, will be fixed in next push.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/mapping.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="108" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB155895-4DD4-420C-A568-B817D6686D14}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CC1269F-0A0F-49AE-89D8-C4A20F4E35C9}"/>
   <bookViews>
-    <workbookView xWindow="4785" yWindow="2940" windowWidth="19290" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3100" yWindow="1870" windowWidth="14400" windowHeight="8180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="45">
   <si>
     <t>sector_from</t>
   </si>
@@ -47,124 +47,130 @@
     <t>sat_accounts</t>
   </si>
   <si>
+    <t>sector_to</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>mario</t>
+  </si>
+  <si>
+    <t>cvxlab</t>
+  </si>
+  <si>
+    <t>Sector_from</t>
+  </si>
+  <si>
+    <t>Sector_to</t>
+  </si>
+  <si>
+    <t>Factor of production_from</t>
+  </si>
+  <si>
+    <t>Satellite account_from</t>
+  </si>
+  <si>
+    <t>Consumption category_to</t>
+  </si>
+  <si>
+    <t>mario flat</t>
+  </si>
+  <si>
+    <t>Sector</t>
+  </si>
+  <si>
+    <t>Factor of production</t>
+  </si>
+  <si>
+    <t>Satellite account</t>
+  </si>
+  <si>
+    <t>Consumption category</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Yold</t>
+  </si>
+  <si>
+    <t>Zold</t>
+  </si>
+  <si>
+    <t>Xnew</t>
+  </si>
+  <si>
+    <t>Ynew0</t>
+  </si>
+  <si>
+    <t>VA</t>
+  </si>
+  <si>
+    <t>Znew0</t>
+  </si>
+  <si>
+    <t>Region_from</t>
+  </si>
+  <si>
+    <t>Region_to</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>region_from</t>
+  </si>
+  <si>
+    <t>region_to</t>
+  </si>
+  <si>
+    <t>cons_categ</t>
+  </si>
+  <si>
+    <t>Znew_supply</t>
+  </si>
+  <si>
+    <t>Znew_use</t>
+  </si>
+  <si>
+    <t>Ynew</t>
+  </si>
+  <si>
+    <t>indeces</t>
+  </si>
+  <si>
+    <t>unstack</t>
+  </si>
+  <si>
+    <t>region_from_Name, sector_from_Name, region_to_Name, sector_to_Name</t>
+  </si>
+  <si>
+    <t>region_from_Name, sector_from_Name, region_to_Name, cons_categ_Name</t>
+  </si>
+  <si>
+    <t>region_to_Name, cons_categ_Name</t>
+  </si>
+  <si>
+    <t>region_to_Name, sector_to_Name</t>
+  </si>
+  <si>
+    <t>Scalar</t>
+  </si>
+  <si>
+    <t>scalar</t>
+  </si>
+  <si>
     <t>scenarios</t>
   </si>
   <si>
-    <t>sector_to</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>mario</t>
-  </si>
-  <si>
-    <t>cvxlab</t>
-  </si>
-  <si>
-    <t>Sector_from</t>
-  </si>
-  <si>
-    <t>Sector_to</t>
-  </si>
-  <si>
-    <t>Factor of production_from</t>
-  </si>
-  <si>
-    <t>Satellite account_from</t>
-  </si>
-  <si>
-    <t>Consumption category_to</t>
-  </si>
-  <si>
     <t>Scenario</t>
-  </si>
-  <si>
-    <t>mario flat</t>
-  </si>
-  <si>
-    <t>Sector</t>
-  </si>
-  <si>
-    <t>Factor of production</t>
-  </si>
-  <si>
-    <t>Satellite account</t>
-  </si>
-  <si>
-    <t>Consumption category</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Yold</t>
-  </si>
-  <si>
-    <t>Zold</t>
-  </si>
-  <si>
-    <t>Xnew</t>
-  </si>
-  <si>
-    <t>Ynew0</t>
-  </si>
-  <si>
-    <t>VA</t>
-  </si>
-  <si>
-    <t>Znew0</t>
-  </si>
-  <si>
-    <t>Region_from</t>
-  </si>
-  <si>
-    <t>Region_to</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>region_from</t>
-  </si>
-  <si>
-    <t>region_to</t>
-  </si>
-  <si>
-    <t>cons_categ</t>
-  </si>
-  <si>
-    <t>Znew_supply</t>
-  </si>
-  <si>
-    <t>Znew_use</t>
-  </si>
-  <si>
-    <t>Ynew</t>
-  </si>
-  <si>
-    <t>indeces</t>
-  </si>
-  <si>
-    <t>unstack</t>
-  </si>
-  <si>
-    <t>region_from_Name, sector_from_Name, region_to_Name, sector_to_Name</t>
-  </si>
-  <si>
-    <t>region_from_Name, sector_from_Name, region_to_Name, cons_categ_Name</t>
-  </si>
-  <si>
-    <t>region_to_Name, cons_categ_Name</t>
-  </si>
-  <si>
-    <t>region_to_Name, sector_to_Name</t>
   </si>
 </sst>
 </file>
@@ -529,111 +535,122 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.54296875" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>3</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -644,61 +661,61 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81EB35F2-9F14-A44D-AA1B-E427820E5706}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -709,39 +726,39 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212F1892-DFA1-4A7F-B6A7-3C40EACDE056}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -752,62 +769,62 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2E9369E-B0C1-4C05-9A69-D044DE2827CA}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improvements in MARIO-cvxlab integration
Implemented possibility to pass parameters to cvxpy solver.
Changes in "Split_sectors" cvxlab problem.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/mapping.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CC1269F-0A0F-49AE-89D8-C4A20F4E35C9}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{881DE90B-C272-4939-929E-36C08BAC7F1A}"/>
   <bookViews>
-    <workbookView xWindow="3100" yWindow="1870" windowWidth="14400" windowHeight="8180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="44">
   <si>
     <t>sector_from</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>Xnew</t>
-  </si>
-  <si>
-    <t>Ynew0</t>
   </si>
   <si>
     <t>VA</t>
@@ -578,24 +575,24 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
         <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -628,29 +625,29 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
         <v>41</v>
-      </c>
-      <c r="B10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -676,10 +673,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
         <v>23</v>
@@ -687,10 +684,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
@@ -698,24 +695,21 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -770,6 +764,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2E9369E-B0C1-4C05-9A69-D044DE2827CA}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -779,52 +776,52 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split sectors: V as a variable
Change of cvxlab to have parent and new values of V as possible variables.

Also, giving new name to the parent sector at the end of disaggregation.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/mapping.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{881DE90B-C272-4939-929E-36C08BAC7F1A}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D6B8CAD-6115-41EF-B177-569B32464BE9}"/>
   <bookViews>
-    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
   <si>
     <t>sector_from</t>
   </si>
@@ -104,15 +104,6 @@
     <t>Zold</t>
   </si>
   <si>
-    <t>Xnew</t>
-  </si>
-  <si>
-    <t>VA</t>
-  </si>
-  <si>
-    <t>Znew0</t>
-  </si>
-  <si>
     <t>Region_from</t>
   </si>
   <si>
@@ -131,15 +122,6 @@
     <t>cons_categ</t>
   </si>
   <si>
-    <t>Znew_supply</t>
-  </si>
-  <si>
-    <t>Znew_use</t>
-  </si>
-  <si>
-    <t>Ynew</t>
-  </si>
-  <si>
     <t>indeces</t>
   </si>
   <si>
@@ -168,6 +150,21 @@
   </si>
   <si>
     <t>Scenario</t>
+  </si>
+  <si>
+    <t>Z0</t>
+  </si>
+  <si>
+    <t>Vold</t>
+  </si>
+  <si>
+    <t>Z_supply</t>
+  </si>
+  <si>
+    <t>Z_use</t>
+  </si>
+  <si>
+    <t>V0</t>
   </si>
 </sst>
 </file>
@@ -575,24 +572,24 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -625,29 +622,29 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -679,7 +676,7 @@
         <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -690,7 +687,7 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -701,7 +698,7 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -719,7 +716,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212F1892-DFA1-4A7F-B6A7-3C40EACDE056}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -755,6 +752,17 @@
         <v>21</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -762,7 +770,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2E9369E-B0C1-4C05-9A69-D044DE2827CA}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -776,55 +784,322 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
+    <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="90e7079a-7589-470d-892b-836f3f5ab9a4" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9ef6bf99-292f-445d-95df-6a8984d5eb85" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{26c05da7-2055-4578-a7cf-40c9d64d09c1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="9ef6bf99-292f-445d-95df-6a8984d5eb85">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7136583B-0E12-4F32-9DC3-CEA66EA1ADA6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF91800-7C7C-4C15-B27A-25CA300FEE60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B73AB652-A38E-40C3-9154-D1AFFD078230}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
2 changes: created AUSteel cvxlab model + Factors of production in Split_sectors
New "default_settings" for cvxlab models: AuSteel, also fixing the db reading part of models.py.
In Split_sector problems now it is possible to define V on multiple rows, the set Factor of Production now is present.
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/Split_sectors/mapping.xlsx
+++ b/mario/tools/cvxlab/Split_sectors/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/Split_sectors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D6B8CAD-6115-41EF-B177-569B32464BE9}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D218C282-1966-43CF-9469-24CF3D0BA3AF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="44">
   <si>
     <t>sector_from</t>
   </si>
   <si>
-    <t>factors</t>
-  </si>
-  <si>
     <t>sat_accounts</t>
   </si>
   <si>
@@ -162,6 +159,12 @@
   </si>
   <si>
     <t>Z_use</t>
+  </si>
+  <si>
+    <t>factor</t>
+  </si>
+  <si>
+    <t>factor_Name, region_to_Name, sector_to_Name</t>
   </si>
   <si>
     <t>V0</t>
@@ -539,21 +542,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
@@ -561,90 +564,90 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>1</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
         <v>34</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -659,54 +662,54 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -721,46 +724,46 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -778,72 +781,72 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -852,8 +855,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="348072715f26cde881c56d84fe7c6dcc">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53f9bc5e977a2cc0a870214cffd63ac6" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
     <xsd:import namespace="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
     <xsd:element name="properties">
@@ -902,7 +914,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Tag immagine" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cb97a35b-a029-4e12-bd78-87cfbccc288e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -956,8 +968,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo di contenuto"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titolo"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -1046,15 +1058,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1067,7 +1070,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7136583B-0E12-4F32-9DC3-CEA66EA1ADA6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF91800-7C7C-4C15-B27A-25CA300FEE60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{182B1835-B6C4-4406-818C-47682B4E6A5C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1085,14 +1096,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CF91800-7C7C-4C15-B27A-25CA300FEE60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B73AB652-A38E-40C3-9154-D1AFFD078230}">
   <ds:schemaRefs>

</xml_diff>